<commit_message>
mdu data 2025 processed
</commit_message>
<xml_diff>
--- a/data/mdu/original_data/mdu_lev7_2025.xlsx
+++ b/data/mdu/original_data/mdu_lev7_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UBA\Medier\OA_artikelkostnad\OA_statistik_KB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/mdu/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13582020-DF92-4D4A-A509-92B8B69E6F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{537E8674-5E3B-5344-AECB-6842F96A6DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{42103501-906A-47D1-9B1C-91744AB20BF8}"/>
+    <workbookView xWindow="74260" yWindow="600" windowWidth="38400" windowHeight="23400" xr2:uid="{42103501-906A-47D1-9B1C-91744AB20BF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="74">
   <si>
     <t>MDPI</t>
   </si>
@@ -246,6 +246,18 @@
   </si>
   <si>
     <t>10.1109/TAES.2025.3646567</t>
+  </si>
+  <si>
+    <t>issn</t>
+  </si>
+  <si>
+    <t>issn_print</t>
+  </si>
+  <si>
+    <t>issn_electronic</t>
+  </si>
+  <si>
+    <t>url</t>
   </si>
 </sst>
 </file>
@@ -297,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -328,16 +340,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -358,9 +360,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -398,7 +400,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -504,7 +506,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -654,19 +656,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184A7841-ED31-45F1-A758-F23998CBB241}">
-  <dimension ref="A1:I30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K30"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.5" customWidth="1"/>
+    <col min="2" max="2" width="9.5" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="37.33203125" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" customWidth="1"/>
     <col min="6" max="6" width="52.6640625" customWidth="1"/>
     <col min="7" max="7" width="71.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -688,8 +690,20 @@
       <c r="G1" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -712,7 +726,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -735,7 +749,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -758,7 +772,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -781,7 +795,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -804,7 +818,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -827,7 +841,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -850,7 +864,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -874,7 +888,7 @@
       </c>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -897,7 +911,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -920,7 +934,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -943,30 +957,30 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="12">
-        <v>2025</v>
-      </c>
-      <c r="C13" s="13">
+    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>2025</v>
+      </c>
+      <c r="C13" s="9">
         <v>7241</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="15" t="s">
+      <c r="E13" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="G13" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>1</v>
       </c>
@@ -989,7 +1003,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -1012,7 +1026,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -1035,7 +1049,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -1058,7 +1072,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -1081,7 +1095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>1</v>
       </c>
@@ -1104,7 +1118,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -1127,7 +1141,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>1</v>
       </c>
@@ -1150,7 +1164,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -1173,7 +1187,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>1</v>
       </c>
@@ -1196,7 +1210,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>1</v>
       </c>
@@ -1219,7 +1233,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -1242,7 +1256,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>1</v>
       </c>
@@ -1265,7 +1279,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>1</v>
       </c>
@@ -1288,7 +1302,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1311,7 +1325,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1334,7 +1348,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>1</v>
       </c>

</xml_diff>